<commit_message>
fix: report screening table field mapping (N/A -> real counts)
_screening_steps_frame fallback used legacy keys absent from refine's stage_summary.json, so the report showed N/A for 原始候选总数 / Feather可用特征 / 最终训练特征. Align to actual keys: initial_features / available_features / final_features. d01/d02 remain N/A in local_feather mode (prescreen by-design). Regression test added.
</commit_message>
<xml_diff>
--- a/projects/2026-05-fujie-gcard-v1/runs/2026-06-30-gcard-main-lgbm-full/reports/model_report.xlsx
+++ b/projects/2026-05-fujie-gcard-v1/runs/2026-06-30-gcard-main-lgbm-full/reports/model_report.xlsx
@@ -24822,10 +24822,8 @@
           <t>原始候选变量总数</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C3" s="7" t="n">
+        <v>2837</v>
       </c>
     </row>
     <row r="4">
@@ -24867,10 +24865,8 @@
           <t>Feather观察样本可用特征</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C6" s="7" t="n">
+        <v>2563</v>
       </c>
     </row>
     <row r="7">
@@ -24921,10 +24917,8 @@
           <t>最终训练特征</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C10" s="7" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="11"/>

</xml_diff>